<commit_message>
Some additions to main text, updated extrapolation data
</commit_message>
<xml_diff>
--- a/exciton.xlsx
+++ b/exciton.xlsx
@@ -136,7 +136,7 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -159,6 +159,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF993300"/>
       </patternFill>
     </fill>
   </fills>
@@ -196,7 +202,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -221,19 +227,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -315,7 +317,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AJ23"/>
-  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1636,7 +1638,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AE18"/>
-  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -2712,7 +2714,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AB20"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -2782,7 +2784,7 @@
       <c r="N3" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="P3" s="0" t="n">
+      <c r="P3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="Q3" s="2" t="n">
@@ -2823,29 +2825,23 @@
       <c r="C4" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
       <c r="J4" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="7"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="7"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
       <c r="Q4" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="R4" s="7"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="7"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
       <c r="X4" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="Y4" s="7"/>
-      <c r="Z4" s="6"/>
-      <c r="AA4" s="6"/>
-      <c r="AB4" s="7"/>
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="0" t="n">
@@ -2854,10 +2850,10 @@
       <c r="D5" s="0" t="n">
         <v>0.4828</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="6" t="n">
         <v>1.8094</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="6" t="n">
         <v>1.8094</v>
       </c>
       <c r="G5" s="0" t="n">
@@ -2873,10 +2869,10 @@
       <c r="K5" s="0" t="n">
         <v>0.4828</v>
       </c>
-      <c r="L5" s="8" t="n">
+      <c r="L5" s="6" t="n">
         <v>1.8094</v>
       </c>
-      <c r="M5" s="8" t="n">
+      <c r="M5" s="6" t="n">
         <v>1.8094</v>
       </c>
       <c r="N5" s="0" t="n">
@@ -2892,10 +2888,10 @@
       <c r="R5" s="0" t="n">
         <v>0.4828</v>
       </c>
-      <c r="S5" s="8" t="n">
+      <c r="S5" s="6" t="n">
         <v>1.8094</v>
       </c>
-      <c r="T5" s="8" t="n">
+      <c r="T5" s="6" t="n">
         <v>1.8094</v>
       </c>
       <c r="U5" s="0" t="n">
@@ -2911,10 +2907,10 @@
       <c r="Y5" s="0" t="n">
         <v>0.4828</v>
       </c>
-      <c r="Z5" s="8" t="n">
+      <c r="Z5" s="6" t="n">
         <v>1.8094</v>
       </c>
-      <c r="AA5" s="8" t="n">
+      <c r="AA5" s="6" t="n">
         <v>1.8094</v>
       </c>
       <c r="AB5" s="0" t="n">
@@ -3107,23 +3103,44 @@
         <v>1.0068</v>
       </c>
     </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P9" s="0" t="n">
+        <f aca="false">COS(3.14159265359/(Q9+1))</f>
+        <v>0.866025403784421</v>
+      </c>
+      <c r="Q9" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="R9" s="0" t="n">
+        <v>1.0974</v>
+      </c>
+      <c r="S9" s="0" t="n">
+        <v>1.8383</v>
+      </c>
+      <c r="T9" s="0" t="n">
+        <v>1.9399</v>
+      </c>
+      <c r="U9" s="0" t="n">
+        <v>1.1062</v>
+      </c>
+    </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L10" s="9" t="n">
+      <c r="L10" s="7" t="n">
         <v>1.8776</v>
       </c>
-      <c r="M10" s="9" t="n">
+      <c r="M10" s="7" t="n">
         <v>1.9444</v>
       </c>
-      <c r="S10" s="9" t="n">
+      <c r="S10" s="8" t="n">
         <v>1.84</v>
       </c>
-      <c r="T10" s="9" t="n">
+      <c r="T10" s="8" t="n">
         <v>1.9554</v>
       </c>
-      <c r="Z10" s="9" t="n">
+      <c r="Z10" s="7" t="n">
         <v>1.8111</v>
       </c>
-      <c r="AA10" s="9" t="n">
+      <c r="AA10" s="7" t="n">
         <v>1.9684</v>
       </c>
     </row>
@@ -3172,16 +3189,20 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0" t="n">
+        <f aca="false">COS(3.14159265359/(C16+1))</f>
+        <v>-1.03411553555107E-013</v>
+      </c>
       <c r="C16" s="0" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="0" t="n">
         <v>0.4828</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="6" t="n">
         <v>1.8094</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="6" t="n">
         <v>1.8094</v>
       </c>
       <c r="G16" s="0" t="n">
@@ -3189,6 +3210,10 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0" t="n">
+        <f aca="false">COS(3.14159265359/(C17+1))</f>
+        <v>0.49999999999994</v>
+      </c>
       <c r="C17" s="0" t="n">
         <v>2</v>
       </c>
@@ -3206,6 +3231,10 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="0" t="n">
+        <f aca="false">COS(3.14159265359/(C18+1))</f>
+        <v>0.707106781186511</v>
+      </c>
       <c r="C18" s="0" t="n">
         <v>3</v>
       </c>
@@ -3223,6 +3252,10 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="0" t="n">
+        <f aca="false">COS(3.14159265359/(C19+1))</f>
+        <v>0.809016994374923</v>
+      </c>
       <c r="C19" s="0" t="n">
         <v>4</v>
       </c>
@@ -3240,6 +3273,10 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="0" t="n">
+        <f aca="false">COS(3.14159265359/(C20+1))</f>
+        <v>0.866025403784421</v>
+      </c>
       <c r="C20" s="0" t="n">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Added values for other shift direction alpha-ZnPc
</commit_message>
<xml_diff>
--- a/exciton.xlsx
+++ b/exciton.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\ms_excitonic\"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="28">
   <si>
     <t>along N-Zn-N</t>
   </si>
@@ -118,7 +118,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -184,14 +184,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -282,10 +282,10 @@
   <a:themeElements>
     <a:clrScheme name="Стандартная">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -323,116 +323,52 @@
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
                 <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
                 <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
                 <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
                 <a:lumMod val="102000"/>
                 <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
                 <a:lumMod val="100000"/>
                 <a:shade val="100000"/>
               </a:schemeClr>
@@ -440,33 +376,24 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
                 <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
@@ -479,13 +406,7 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -495,15 +416,13 @@
         <a:solidFill>
           <a:schemeClr val="phClr">
             <a:tint val="95000"/>
-            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
               </a:schemeClr>
@@ -511,7 +430,6 @@
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
               </a:schemeClr>
@@ -519,22 +437,17 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="63000"/>
-                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -2929,7 +2842,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB44"/>
+  <dimension ref="A1:AB47"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.2">
@@ -3441,16 +3354,16 @@
       <c r="C16" s="3">
         <v>1</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="11">
         <v>0.47199999999999998</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="F16" s="13">
+      <c r="F16" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="11">
         <v>0.47199999999999998</v>
       </c>
       <c r="P16" s="3">
@@ -3481,16 +3394,16 @@
       <c r="C17" s="3">
         <v>2</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="13">
         <v>0.6845</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="13">
         <v>1.7946</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="13">
         <v>1.9097999999999999</v>
       </c>
-      <c r="G17" s="14">
+      <c r="G17" s="13">
         <v>0.66769999999999996</v>
       </c>
       <c r="P17" s="3">
@@ -3521,16 +3434,16 @@
       <c r="C18" s="3">
         <v>3</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="13">
         <v>0.95720000000000005</v>
       </c>
-      <c r="E18" s="14">
+      <c r="E18" s="13">
         <v>1.7791999999999999</v>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="13">
         <v>1.9390000000000001</v>
       </c>
-      <c r="G18" s="14">
+      <c r="G18" s="13">
         <v>0.82569999999999999</v>
       </c>
       <c r="P18" s="3">
@@ -3561,16 +3474,16 @@
       <c r="C19" s="3">
         <v>4</v>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="13">
         <v>1.2312000000000001</v>
       </c>
-      <c r="E19" s="14">
+      <c r="E19" s="13">
         <v>1.7698</v>
       </c>
-      <c r="F19" s="14">
+      <c r="F19" s="13">
         <v>1.9551000000000001</v>
       </c>
-      <c r="G19" s="14">
+      <c r="G19" s="13">
         <v>0.9728</v>
       </c>
       <c r="P19" s="3">
@@ -3601,16 +3514,16 @@
       <c r="C20" s="3">
         <v>5</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="11">
         <v>1.4281999999999999</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="11">
         <v>1.7645</v>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="11">
         <v>1.9653</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="11">
         <v>1.1142000000000001</v>
       </c>
       <c r="R20" s="8">
@@ -3624,22 +3537,22 @@
       </c>
     </row>
     <row r="21" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="D21" s="15">
+      <c r="D21" s="14">
         <v>1.5469999999999999</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="14">
         <v>1.7524</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="14">
         <v>1.9819</v>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="15">
         <v>1</v>
       </c>
       <c r="S21" s="9">
         <v>1.8030999999999999</v>
       </c>
-      <c r="T21" s="11">
+      <c r="T21" s="16">
         <v>1.9291</v>
       </c>
     </row>
@@ -3719,6 +3632,12 @@
       <c r="AA27" s="5"/>
     </row>
     <row r="28" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="P28" s="3">
         <f>COS(3.14159265359/(Q28+1))</f>
         <v>-1.0341152847231916E-13</v>
@@ -3726,16 +3645,16 @@
       <c r="Q28" s="3">
         <v>1</v>
       </c>
-      <c r="R28" s="12">
+      <c r="R28" s="11">
         <v>0.47199999999999998</v>
       </c>
-      <c r="S28" s="13">
+      <c r="S28" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="T28" s="13">
+      <c r="T28" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="U28" s="12">
+      <c r="U28" s="11">
         <v>0.47199999999999998</v>
       </c>
       <c r="W28" s="3">
@@ -3745,20 +3664,38 @@
       <c r="X28" s="3">
         <v>1</v>
       </c>
-      <c r="Y28" s="12">
+      <c r="Y28" s="11">
         <v>0.47199999999999998</v>
       </c>
-      <c r="Z28" s="13">
+      <c r="Z28" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="AA28" s="13">
+      <c r="AA28" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="AB28" s="12">
+      <c r="AB28" s="11">
         <v>0.47199999999999998</v>
       </c>
     </row>
     <row r="29" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B29" s="2">
+        <v>2</v>
+      </c>
+      <c r="C29" s="2">
+        <v>3.4</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="P29" s="3">
         <f>COS(3.14159265359/(Q29+1))</f>
         <v>0.49999999999994027</v>
@@ -3766,16 +3703,16 @@
       <c r="Q29" s="3">
         <v>2</v>
       </c>
-      <c r="R29" s="14">
+      <c r="R29" s="13">
         <v>0.56259999999999999</v>
       </c>
-      <c r="S29" s="14">
+      <c r="S29" s="13">
         <v>1.8226</v>
       </c>
-      <c r="T29" s="14">
+      <c r="T29" s="13">
         <v>1.9006000000000001</v>
       </c>
-      <c r="U29" s="14">
+      <c r="U29" s="13">
         <v>0.62329999999999997</v>
       </c>
       <c r="W29" s="3">
@@ -3785,20 +3722,25 @@
       <c r="X29" s="3">
         <v>2</v>
       </c>
-      <c r="Y29" s="14">
+      <c r="Y29" s="13">
         <v>0.52080000000000004</v>
       </c>
-      <c r="Z29" s="14">
+      <c r="Z29" s="13">
         <v>1.7909999999999999</v>
       </c>
-      <c r="AA29" s="14">
+      <c r="AA29" s="13">
         <v>1.8908</v>
       </c>
-      <c r="AB29" s="14">
+      <c r="AB29" s="13">
         <v>0.59809999999999997</v>
       </c>
     </row>
     <row r="30" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="C30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
       <c r="P30" s="3">
         <f>COS(3.14159265359/(Q30+1))</f>
         <v>0.70710678118651094</v>
@@ -3806,16 +3748,16 @@
       <c r="Q30" s="3">
         <v>3</v>
       </c>
-      <c r="R30" s="14">
+      <c r="R30" s="13">
         <v>0.6794</v>
       </c>
-      <c r="S30" s="14">
+      <c r="S30" s="13">
         <v>1.8207</v>
       </c>
-      <c r="T30" s="14">
+      <c r="T30" s="13">
         <v>1.9256</v>
       </c>
-      <c r="U30" s="14">
+      <c r="U30" s="13">
         <v>0.75419999999999998</v>
       </c>
       <c r="W30" s="3">
@@ -3825,20 +3767,39 @@
       <c r="X30" s="3">
         <v>3</v>
       </c>
-      <c r="Y30" s="14">
+      <c r="Y30" s="13">
         <v>0.61819999999999997</v>
       </c>
-      <c r="Z30" s="14">
+      <c r="Z30" s="13">
         <v>1.7823</v>
       </c>
-      <c r="AA30" s="14">
+      <c r="AA30" s="13">
         <v>1.9121999999999999</v>
       </c>
-      <c r="AB30" s="14">
+      <c r="AB30" s="13">
         <v>0.71540000000000004</v>
       </c>
     </row>
     <row r="31" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B31" s="3">
+        <f>COS(3.14159265359/(C31+1))</f>
+        <v>-1.0341152847231916E-13</v>
+      </c>
+      <c r="C31" s="3">
+        <v>1</v>
+      </c>
+      <c r="D31" s="11">
+        <v>0.47199999999999998</v>
+      </c>
+      <c r="E31" s="12">
+        <v>1.8420000000000001</v>
+      </c>
+      <c r="F31" s="12">
+        <v>1.8420000000000001</v>
+      </c>
+      <c r="G31" s="11">
+        <v>0.47199999999999998</v>
+      </c>
       <c r="P31" s="3">
         <f>COS(3.14159265359/(Q31+1))</f>
         <v>0.80901699437492314</v>
@@ -3846,16 +3807,16 @@
       <c r="Q31" s="3">
         <v>4</v>
       </c>
-      <c r="R31" s="14">
+      <c r="R31" s="13">
         <v>0.80520000000000003</v>
       </c>
-      <c r="S31" s="14">
+      <c r="S31" s="13">
         <v>1.82</v>
       </c>
-      <c r="T31" s="14">
+      <c r="T31" s="13">
         <v>1.9390000000000001</v>
       </c>
-      <c r="U31" s="14">
+      <c r="U31" s="13">
         <v>0.88119999999999998</v>
       </c>
       <c r="W31" s="3">
@@ -3865,51 +3826,129 @@
       <c r="X31" s="3">
         <v>4</v>
       </c>
-      <c r="Y31" s="14">
+      <c r="Y31" s="13">
         <v>0.73040000000000005</v>
       </c>
-      <c r="Z31" s="14">
+      <c r="Z31" s="13">
         <v>1.778</v>
       </c>
-      <c r="AA31" s="14">
+      <c r="AA31" s="13">
         <v>1.9235</v>
       </c>
-      <c r="AB31" s="14">
+      <c r="AB31" s="13">
         <v>0.82769999999999999</v>
       </c>
     </row>
     <row r="32" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="R32" s="18">
+      <c r="B32" s="3">
+        <f>COS(3.14159265359/(C32+1))</f>
+        <v>0.49999999999994027</v>
+      </c>
+      <c r="C32" s="3">
+        <v>2</v>
+      </c>
+      <c r="D32" s="13">
+        <v>0.68330000000000002</v>
+      </c>
+      <c r="E32" s="13">
+        <v>1.8963000000000001</v>
+      </c>
+      <c r="F32" s="13">
+        <v>1.8995</v>
+      </c>
+      <c r="G32" s="13">
+        <v>0.60629999999999995</v>
+      </c>
+      <c r="R32" s="17">
         <v>1</v>
       </c>
-      <c r="S32" s="15">
+      <c r="S32" s="14">
         <v>1.8123</v>
       </c>
-      <c r="T32" s="15">
+      <c r="T32" s="14">
         <v>1.9610000000000001</v>
       </c>
-      <c r="U32" s="15">
+      <c r="U32" s="14">
         <v>1.2170000000000001</v>
       </c>
-      <c r="Y32" s="18">
+      <c r="Y32" s="17">
         <v>1</v>
       </c>
-      <c r="Z32" s="17">
+      <c r="Z32" s="18">
         <v>1.7582</v>
       </c>
-      <c r="AA32" s="17">
+      <c r="AA32" s="18">
         <v>1.9418</v>
       </c>
-      <c r="AB32" s="17">
+      <c r="AB32" s="18">
         <v>1.357</v>
       </c>
     </row>
-    <row r="33" spans="16:28" x14ac:dyDescent="0.2">
-      <c r="S33" s="9"/>
-      <c r="T33" s="9"/>
-      <c r="U33" s="9"/>
-    </row>
-    <row r="37" spans="16:28" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B33" s="3">
+        <f>COS(3.14159265359/(C33+1))</f>
+        <v>0.70710678118651094</v>
+      </c>
+      <c r="C33" s="3">
+        <v>3</v>
+      </c>
+      <c r="D33" s="13">
+        <v>0.87429999999999997</v>
+      </c>
+      <c r="E33" s="13">
+        <v>1.9197</v>
+      </c>
+      <c r="F33" s="13">
+        <v>1.9226000000000001</v>
+      </c>
+      <c r="G33" s="13">
+        <v>0.70530000000000004</v>
+      </c>
+      <c r="S33" s="3"/>
+      <c r="T33" s="3"/>
+      <c r="U33" s="3"/>
+    </row>
+    <row r="34" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B34" s="3">
+        <f>COS(3.14159265359/(C34+1))</f>
+        <v>0.80901699437492314</v>
+      </c>
+      <c r="C34" s="3">
+        <v>4</v>
+      </c>
+      <c r="D34" s="13">
+        <v>1.0605</v>
+      </c>
+      <c r="E34" s="13">
+        <v>1.9320999999999999</v>
+      </c>
+      <c r="F34" s="13">
+        <v>1.9347000000000001</v>
+      </c>
+      <c r="G34" s="13">
+        <v>0.79759999999999998</v>
+      </c>
+    </row>
+    <row r="35" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="D35" s="18">
+        <v>1.819</v>
+      </c>
+      <c r="E35" s="14">
+        <v>1.9524999999999999</v>
+      </c>
+      <c r="F35" s="14">
+        <v>1.9563999999999999</v>
+      </c>
+      <c r="G35" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+    </row>
+    <row r="37" spans="2:28" x14ac:dyDescent="0.2">
       <c r="P37" s="3" t="s">
         <v>9</v>
       </c>
@@ -3923,7 +3962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="16:28" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:28" x14ac:dyDescent="0.2">
       <c r="P38" s="10">
         <v>1.75</v>
       </c>
@@ -3961,7 +4000,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="16:28" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:28" x14ac:dyDescent="0.2">
       <c r="Q39" s="3" t="s">
         <v>19</v>
       </c>
@@ -3973,7 +4012,13 @@
       <c r="Z39" s="5"/>
       <c r="AA39" s="5"/>
     </row>
-    <row r="40" spans="16:28" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B40" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="P40" s="3">
         <f>COS(3.14159265359/(Q40+1))</f>
         <v>-1.0341152847231916E-13</v>
@@ -3981,16 +4026,16 @@
       <c r="Q40" s="3">
         <v>1</v>
       </c>
-      <c r="R40" s="12">
+      <c r="R40" s="11">
         <v>0.47199999999999998</v>
       </c>
-      <c r="S40" s="13">
+      <c r="S40" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="T40" s="13">
+      <c r="T40" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="U40" s="12">
+      <c r="U40" s="11">
         <v>0.47199999999999998</v>
       </c>
       <c r="W40" s="3">
@@ -4000,20 +4045,38 @@
       <c r="X40" s="3">
         <v>1</v>
       </c>
-      <c r="Y40" s="12">
+      <c r="Y40" s="11">
         <v>0.47199999999999998</v>
       </c>
-      <c r="Z40" s="13">
+      <c r="Z40" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="AA40" s="13">
+      <c r="AA40" s="12">
         <v>1.8420000000000001</v>
       </c>
-      <c r="AB40" s="12">
+      <c r="AB40" s="11">
         <v>0.47199999999999998</v>
       </c>
     </row>
-    <row r="41" spans="16:28" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B41" s="10">
+        <v>1.75</v>
+      </c>
+      <c r="C41" s="2">
+        <v>3.4</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="P41" s="3">
         <f>COS(3.14159265359/(Q41+1))</f>
         <v>0.49999999999994027</v>
@@ -4021,16 +4084,16 @@
       <c r="Q41" s="3">
         <v>2</v>
       </c>
-      <c r="R41" s="14">
+      <c r="R41" s="13">
         <v>0.56810000000000005</v>
       </c>
-      <c r="S41" s="14">
+      <c r="S41" s="13">
         <v>1.8462000000000001</v>
       </c>
-      <c r="T41" s="14">
+      <c r="T41" s="13">
         <v>1.8887</v>
       </c>
-      <c r="U41" s="14">
+      <c r="U41" s="13">
         <v>0.59860000000000002</v>
       </c>
       <c r="W41" s="3">
@@ -4040,20 +4103,25 @@
       <c r="X41" s="3">
         <v>2</v>
       </c>
-      <c r="Y41" s="14">
+      <c r="Y41" s="13">
         <v>0.5242</v>
       </c>
-      <c r="Z41" s="14">
+      <c r="Z41" s="13">
         <v>1.8202</v>
       </c>
-      <c r="AA41" s="14">
+      <c r="AA41" s="13">
         <v>1.8723000000000001</v>
       </c>
-      <c r="AB41" s="14">
+      <c r="AB41" s="13">
         <v>0.56389999999999996</v>
       </c>
     </row>
-    <row r="42" spans="16:28" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="C42" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
       <c r="P42" s="3">
         <f>COS(3.14159265359/(Q42+1))</f>
         <v>0.70710678118651094</v>
@@ -4061,16 +4129,16 @@
       <c r="Q42" s="3">
         <v>3</v>
       </c>
-      <c r="R42" s="14">
+      <c r="R42" s="13">
         <v>0.68169999999999997</v>
       </c>
-      <c r="S42" s="14">
+      <c r="S42" s="13">
         <v>1.8543000000000001</v>
       </c>
-      <c r="T42" s="14">
+      <c r="T42" s="13">
         <v>1.91</v>
       </c>
-      <c r="U42" s="14">
+      <c r="U42" s="13">
         <v>0.71209999999999996</v>
       </c>
       <c r="W42" s="3">
@@ -4080,20 +4148,39 @@
       <c r="X42" s="3">
         <v>3</v>
       </c>
-      <c r="Y42" s="14">
+      <c r="Y42" s="13">
         <v>0.62319999999999998</v>
       </c>
-      <c r="Z42" s="14">
+      <c r="Z42" s="13">
         <v>1.8237000000000001</v>
       </c>
-      <c r="AA42" s="14">
+      <c r="AA42" s="13">
         <v>1.8889</v>
       </c>
-      <c r="AB42" s="14">
+      <c r="AB42" s="13">
         <v>0.66220000000000001</v>
       </c>
     </row>
-    <row r="43" spans="16:28" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B43" s="3">
+        <f>COS(3.14159265359/(C43+1))</f>
+        <v>-1.0341152847231916E-13</v>
+      </c>
+      <c r="C43" s="3">
+        <v>1</v>
+      </c>
+      <c r="D43" s="11">
+        <v>0.47199999999999998</v>
+      </c>
+      <c r="E43" s="12">
+        <v>1.8420000000000001</v>
+      </c>
+      <c r="F43" s="12">
+        <v>1.8420000000000001</v>
+      </c>
+      <c r="G43" s="11">
+        <v>0.47199999999999998</v>
+      </c>
       <c r="P43" s="3">
         <f>COS(3.14159265359/(Q43+1))</f>
         <v>0.80901699437492314</v>
@@ -4101,16 +4188,16 @@
       <c r="Q43" s="3">
         <v>4</v>
       </c>
-      <c r="R43" s="14">
+      <c r="R43" s="13">
         <v>0.7954</v>
       </c>
-      <c r="S43" s="14">
+      <c r="S43" s="13">
         <v>1.8586</v>
       </c>
-      <c r="T43" s="14">
+      <c r="T43" s="13">
         <v>1.9213</v>
       </c>
-      <c r="U43" s="14">
+      <c r="U43" s="13">
         <v>0.8206</v>
       </c>
       <c r="W43" s="3">
@@ -4120,43 +4207,118 @@
       <c r="X43" s="3">
         <v>4</v>
       </c>
-      <c r="Y43" s="14">
+      <c r="Y43" s="13">
         <v>0.72309999999999997</v>
       </c>
-      <c r="Z43" s="14">
+      <c r="Z43" s="13">
         <v>1.8249</v>
       </c>
-      <c r="AA43" s="14">
+      <c r="AA43" s="13">
         <v>1.8973</v>
       </c>
-      <c r="AB43" s="14">
+      <c r="AB43" s="13">
         <v>0.75609999999999999</v>
       </c>
     </row>
-    <row r="44" spans="16:28" x14ac:dyDescent="0.2">
-      <c r="R44" s="18">
+    <row r="44" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B44" s="3">
+        <f>COS(3.14159265359/(C44+1))</f>
+        <v>0.49999999999994027</v>
+      </c>
+      <c r="C44" s="3">
+        <v>2</v>
+      </c>
+      <c r="D44" s="13">
+        <v>0.68330000000000002</v>
+      </c>
+      <c r="E44" s="13">
+        <v>1.8963000000000001</v>
+      </c>
+      <c r="F44" s="13">
+        <v>1.8995</v>
+      </c>
+      <c r="G44" s="13">
+        <v>0.60629999999999995</v>
+      </c>
+      <c r="R44" s="17">
         <v>1</v>
       </c>
-      <c r="S44" s="17">
+      <c r="S44" s="18">
         <v>1.8599000000000001</v>
       </c>
-      <c r="T44" s="17">
+      <c r="T44" s="18">
         <v>1.9388000000000001</v>
       </c>
-      <c r="U44" s="17">
+      <c r="U44" s="18">
         <v>1.07</v>
       </c>
-      <c r="Y44" s="17">
+      <c r="Y44" s="18">
         <v>1</v>
       </c>
-      <c r="Z44" s="17">
+      <c r="Z44" s="18">
         <v>1.8164</v>
       </c>
-      <c r="AA44" s="17">
+      <c r="AA44" s="18">
         <v>1.9087000000000001</v>
       </c>
-      <c r="AB44" s="17">
+      <c r="AB44" s="18">
         <v>1.115</v>
+      </c>
+    </row>
+    <row r="45" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B45" s="3">
+        <f>COS(3.14159265359/(C45+1))</f>
+        <v>0.70710678118651094</v>
+      </c>
+      <c r="C45" s="3">
+        <v>3</v>
+      </c>
+      <c r="D45" s="13">
+        <v>0.85880000000000001</v>
+      </c>
+      <c r="E45" s="13">
+        <v>1.9279999999999999</v>
+      </c>
+      <c r="F45" s="13">
+        <v>1.9297</v>
+      </c>
+      <c r="G45" s="13">
+        <v>0.70550000000000002</v>
+      </c>
+    </row>
+    <row r="46" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="B46" s="3">
+        <f>COS(3.14159265359/(C46+1))</f>
+        <v>0.80901699437492314</v>
+      </c>
+      <c r="C46" s="3">
+        <v>4</v>
+      </c>
+      <c r="D46" s="13">
+        <v>1.0357000000000001</v>
+      </c>
+      <c r="E46" s="13">
+        <v>1.9426000000000001</v>
+      </c>
+      <c r="F46" s="13">
+        <v>1.9429000000000001</v>
+      </c>
+      <c r="G46" s="13">
+        <v>0.78949999999999998</v>
+      </c>
+    </row>
+    <row r="47" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="D47" s="18">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="E47" s="18">
+        <v>1.9630000000000001</v>
+      </c>
+      <c r="F47" s="18">
+        <v>1.9650000000000001</v>
+      </c>
+      <c r="G47" s="17">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>